<commit_message>
Updates for Phase 2
</commit_message>
<xml_diff>
--- a/data/to-migrate/mapping/Professional Actitivies Choice Lists.xlsx
+++ b/data/to-migrate/mapping/Professional Actitivies Choice Lists.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dsmith/Documents/code/lyterati-elements/data/to-migrate/mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8126C662-63A1-5746-AAFE-806DEAF23D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5004663-8675-634D-862F-18DCC9C2A026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{981C8887-6331-42CE-8691-63AB4AAAF8BA}"/>
+    <workbookView xWindow="-32320" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{981C8887-6331-42CE-8691-63AB4AAAF8BA}"/>
   </bookViews>
   <sheets>
     <sheet name="c-membership-type" sheetId="2" r:id="rId1"/>
+    <sheet name="committee-role" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>Academic</t>
   </si>
@@ -57,18 +58,57 @@
   </si>
   <si>
     <t>Elements</t>
+  </si>
+  <si>
+    <t>Lyterati</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>Member</t>
+  </si>
+  <si>
+    <t>Organizer</t>
+  </si>
+  <si>
+    <t>Vice Chair</t>
+  </si>
+  <si>
+    <t>Vice chair</t>
+  </si>
+  <si>
+    <t>Co-Chair</t>
+  </si>
+  <si>
+    <t>Co-chair</t>
+  </si>
+  <si>
+    <t>Vice-President</t>
+  </si>
+  <si>
+    <t>Vice president</t>
+  </si>
+  <si>
+    <t>Senior Member</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -92,8 +132,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,4 +513,86 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C2A1EE-4F83-7C44-BD41-85DFC171121A}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>